<commit_message>
style: modify AIR template for Export feature
</commit_message>
<xml_diff>
--- a/procurement_documents/IAR Template.xlsx
+++ b/procurement_documents/IAR Template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35D3CEF-CDD5-49CF-838F-497EA63AF908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72B7176D-5D01-4F81-A7F9-0680C23A1DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{6CD071E1-92CF-4D3E-842E-C4264179AD1A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{6CD071E1-92CF-4D3E-842E-C4264179AD1A}"/>
   </bookViews>
   <sheets>
     <sheet name="IAR" sheetId="2" r:id="rId1"/>
@@ -579,48 +579,6 @@
   </cellStyleXfs>
   <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -653,9 +611,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -692,15 +647,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -771,6 +717,68 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -780,59 +788,51 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -856,6 +856,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="PAR"/>
@@ -1194,500 +1195,501 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9C83917-B674-4037-AFDD-3840452F802F}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A2:K18099"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="1" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="92" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4" t="s">
+      <c r="B3" s="94"/>
+      <c r="C3" s="94"/>
+      <c r="D3" s="95" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6" t="s">
+      <c r="A4" s="85"/>
+      <c r="B4" s="85"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="96" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="8"/>
+      <c r="E4" s="97"/>
+      <c r="F4" s="98"/>
     </row>
     <row r="5" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="85" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="11"/>
+      <c r="B5" s="85"/>
+      <c r="C5" s="85"/>
+      <c r="D5" s="86"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="88"/>
     </row>
     <row r="6" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="85" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="12" t="s">
+      <c r="B6" s="85"/>
+      <c r="C6" s="85"/>
+      <c r="D6" s="89" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
+      <c r="E6" s="89"/>
+      <c r="F6" s="89"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
+      <c r="B7" s="90"/>
+      <c r="C7" s="90"/>
+      <c r="D7" s="91"/>
+      <c r="E7" s="91"/>
+      <c r="F7" s="91"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="18"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="20"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23" t="s">
+      <c r="B9" s="6"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="24"/>
+      <c r="F9" s="10"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="17" t="s">
+      <c r="B10" s="11"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="27"/>
+      <c r="F10" s="13"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="17" t="s">
+      <c r="B11" s="3"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="29"/>
+      <c r="F11" s="15"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="31"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="31" t="s">
+      <c r="B12" s="17"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="27"/>
+      <c r="F12" s="13"/>
     </row>
     <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="33"/>
-      <c r="D13" s="33"/>
-      <c r="E13" s="34" t="s">
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="34" t="s">
+      <c r="F13" s="19" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="35"/>
-      <c r="B14" s="36"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="35"/>
-      <c r="B15" s="36"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="35"/>
-      <c r="B16" s="41"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="H16" s="98"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="H16" s="67"/>
     </row>
     <row r="17" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="35"/>
-      <c r="B17" s="44"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
+      <c r="A17" s="20"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
     </row>
     <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="35"/>
-      <c r="B18" s="41"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="45"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="30"/>
     </row>
     <row r="19" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="35"/>
-      <c r="B19" s="46"/>
-      <c r="C19" s="42"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="45"/>
+      <c r="A19" s="20"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="30"/>
     </row>
     <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
-      <c r="B20" s="48"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="50"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="45"/>
-      <c r="I20" s="98"/>
+      <c r="A20" s="32"/>
+      <c r="B20" s="78"/>
+      <c r="C20" s="79"/>
+      <c r="D20" s="80"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="30"/>
+      <c r="I20" s="67"/>
     </row>
     <row r="21" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="47"/>
-      <c r="B21" s="51"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="45"/>
-      <c r="K21" s="98"/>
+      <c r="A21" s="32"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="30"/>
+      <c r="K21" s="67"/>
     </row>
     <row r="22" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="47"/>
-      <c r="B22" s="48"/>
-      <c r="C22" s="49"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="54"/>
+      <c r="A22" s="32"/>
+      <c r="B22" s="78"/>
+      <c r="C22" s="79"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="36"/>
     </row>
     <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="47"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
+      <c r="A23" s="32"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
     </row>
     <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="35"/>
-      <c r="B24" s="57"/>
-      <c r="C24" s="58"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="39"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
     </row>
     <row r="25" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="35"/>
-      <c r="B25" s="57"/>
-      <c r="C25" s="58"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="59"/>
+      <c r="A25" s="20"/>
+      <c r="B25" s="39"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="41"/>
     </row>
     <row r="26" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="35"/>
-      <c r="B26" s="36"/>
-      <c r="C26" s="52"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="59"/>
+      <c r="A26" s="20"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="41"/>
     </row>
     <row r="27" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="35"/>
-      <c r="B27" s="36"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="56"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="60"/>
+      <c r="A27" s="20"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="42"/>
     </row>
     <row r="28" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="35"/>
-      <c r="B28" s="36"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="60"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="42"/>
     </row>
     <row r="29" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="35"/>
-      <c r="B29" s="51"/>
-      <c r="C29" s="61"/>
-      <c r="D29" s="40"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="60"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="33"/>
+      <c r="C29" s="43"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="42"/>
     </row>
     <row r="30" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="35"/>
-      <c r="B30" s="51"/>
-      <c r="C30" s="61"/>
-      <c r="D30" s="56"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="60"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="33"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="42"/>
     </row>
     <row r="31" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="35"/>
-      <c r="B31" s="36"/>
-      <c r="C31" s="61"/>
-      <c r="D31" s="56"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="60"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="42"/>
     </row>
     <row r="32" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="35"/>
-      <c r="B32" s="51"/>
-      <c r="C32" s="61"/>
-      <c r="D32" s="62"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="60"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="33"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="42"/>
     </row>
     <row r="33" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="35"/>
-      <c r="B33" s="36"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="39"/>
-      <c r="F33" s="60"/>
+      <c r="A33" s="20"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="42"/>
     </row>
     <row r="34" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="35"/>
-      <c r="B34" s="48"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="50"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="63"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="78"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="80"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="45"/>
     </row>
     <row r="35" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="35"/>
-      <c r="B35" s="64"/>
-      <c r="C35" s="65"/>
-      <c r="D35" s="66"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="67"/>
+      <c r="A35" s="20"/>
+      <c r="B35" s="46"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="49"/>
     </row>
     <row r="36" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="35"/>
-      <c r="B36" s="68"/>
-      <c r="C36" s="69"/>
-      <c r="D36" s="70"/>
-      <c r="E36" s="71"/>
-      <c r="F36" s="67"/>
+      <c r="A36" s="20"/>
+      <c r="B36" s="50"/>
+      <c r="C36" s="51"/>
+      <c r="D36" s="52"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="49"/>
     </row>
     <row r="37" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="35"/>
-      <c r="B37" s="72"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="70"/>
-      <c r="E37" s="39"/>
-      <c r="F37" s="67"/>
+      <c r="A37" s="20"/>
+      <c r="B37" s="54"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="52"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="49"/>
     </row>
     <row r="38" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="35"/>
-      <c r="B38" s="73"/>
-      <c r="C38" s="74"/>
-      <c r="D38" s="38"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="45"/>
+      <c r="A38" s="20"/>
+      <c r="B38" s="55"/>
+      <c r="C38" s="56"/>
+      <c r="D38" s="23"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="30"/>
     </row>
     <row r="39" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="35"/>
-      <c r="B39" s="36"/>
-      <c r="C39" s="75"/>
-      <c r="D39" s="70"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="45"/>
+      <c r="A39" s="20"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="57"/>
+      <c r="D39" s="52"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="30"/>
     </row>
     <row r="40" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="35"/>
-      <c r="B40" s="76"/>
-      <c r="C40" s="75"/>
-      <c r="D40" s="70"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="45"/>
+      <c r="A40" s="20"/>
+      <c r="B40" s="58"/>
+      <c r="C40" s="57"/>
+      <c r="D40" s="52"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="30"/>
     </row>
     <row r="41" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="35"/>
-      <c r="B41" s="77"/>
-      <c r="C41" s="78"/>
-      <c r="D41" s="79"/>
-      <c r="E41" s="80"/>
-      <c r="F41" s="81"/>
+      <c r="A41" s="20"/>
+      <c r="B41" s="81"/>
+      <c r="C41" s="82"/>
+      <c r="D41" s="83"/>
+      <c r="E41" s="59"/>
+      <c r="F41" s="60"/>
     </row>
     <row r="42" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="35"/>
-      <c r="B42" s="82"/>
-      <c r="C42" s="75"/>
-      <c r="D42" s="70"/>
-      <c r="E42" s="80"/>
-      <c r="F42" s="81"/>
+      <c r="A42" s="20"/>
+      <c r="B42" s="61"/>
+      <c r="C42" s="57"/>
+      <c r="D42" s="52"/>
+      <c r="E42" s="59"/>
+      <c r="F42" s="60"/>
     </row>
     <row r="43" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="83" t="s">
+      <c r="A43" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="B43" s="83"/>
-      <c r="C43" s="83"/>
-      <c r="D43" s="83" t="s">
+      <c r="B43" s="84"/>
+      <c r="C43" s="84"/>
+      <c r="D43" s="84" t="s">
         <v>21</v>
       </c>
-      <c r="E43" s="83"/>
-      <c r="F43" s="83"/>
+      <c r="E43" s="84"/>
+      <c r="F43" s="84"/>
     </row>
     <row r="44" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="84"/>
-      <c r="B44" s="85"/>
-      <c r="C44" s="86"/>
-      <c r="D44" s="85"/>
-      <c r="E44" s="85"/>
-      <c r="F44" s="86"/>
+      <c r="A44" s="62"/>
+      <c r="B44" s="63"/>
+      <c r="C44" s="64"/>
+      <c r="D44" s="63"/>
+      <c r="E44" s="63"/>
+      <c r="F44" s="64"/>
     </row>
     <row r="45" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="15" t="s">
+      <c r="A45" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B45" s="26"/>
-      <c r="C45" s="18"/>
-      <c r="D45" s="17" t="s">
+      <c r="B45" s="12"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E45" s="26"/>
-      <c r="F45" s="87"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="65"/>
     </row>
     <row r="46" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
-      <c r="B46" s="17"/>
-      <c r="C46" s="18"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="18"/>
+      <c r="A46" s="1"/>
+      <c r="B46" s="3"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="4"/>
     </row>
     <row r="47" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="88" t="s">
+      <c r="A47" s="71" t="s">
         <v>24</v>
       </c>
-      <c r="B47" s="89"/>
-      <c r="C47" s="90"/>
-      <c r="D47" s="91" t="s">
+      <c r="B47" s="72"/>
+      <c r="C47" s="73"/>
+      <c r="D47" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="E47" s="91" t="s">
+      <c r="E47" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="F47" s="18"/>
+      <c r="F47" s="4"/>
     </row>
     <row r="48" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="88" t="s">
+      <c r="A48" s="71" t="s">
         <v>27</v>
       </c>
-      <c r="B48" s="89"/>
-      <c r="C48" s="90"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17" t="s">
+      <c r="B48" s="72"/>
+      <c r="C48" s="73"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F48" s="18"/>
+      <c r="F48" s="4"/>
     </row>
     <row r="49" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="15"/>
-      <c r="B49" s="17"/>
-      <c r="C49" s="18"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="18"/>
+      <c r="A49" s="1"/>
+      <c r="B49" s="3"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="4"/>
     </row>
     <row r="50" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="15"/>
-      <c r="B50" s="17"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="17"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="18"/>
+      <c r="A50" s="1"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="4"/>
     </row>
     <row r="51" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="92"/>
-      <c r="B51" s="93"/>
-      <c r="C51" s="94"/>
-      <c r="D51" s="93" t="s">
+      <c r="A51" s="74"/>
+      <c r="B51" s="75"/>
+      <c r="C51" s="76"/>
+      <c r="D51" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="E51" s="93"/>
-      <c r="F51" s="94"/>
+      <c r="E51" s="75"/>
+      <c r="F51" s="76"/>
     </row>
     <row r="52" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="88" t="s">
+      <c r="A52" s="71" t="s">
         <v>30</v>
       </c>
-      <c r="B52" s="89"/>
-      <c r="C52" s="90"/>
-      <c r="D52" s="89" t="s">
+      <c r="B52" s="72"/>
+      <c r="C52" s="73"/>
+      <c r="D52" s="72" t="s">
         <v>31</v>
       </c>
-      <c r="E52" s="89"/>
-      <c r="F52" s="90"/>
+      <c r="E52" s="72"/>
+      <c r="F52" s="73"/>
     </row>
     <row r="53" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="95"/>
-      <c r="B53" s="96"/>
-      <c r="C53" s="97"/>
-      <c r="D53" s="96"/>
-      <c r="E53" s="96"/>
-      <c r="F53" s="97"/>
+      <c r="A53" s="68"/>
+      <c r="B53" s="69"/>
+      <c r="C53" s="70"/>
+      <c r="D53" s="69"/>
+      <c r="E53" s="69"/>
+      <c r="F53" s="70"/>
     </row>
     <row r="54" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3817,6 +3819,25 @@
     <row r="18099" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="D43:F43"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B41:D41"/>
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="D53:F53"/>
     <mergeCell ref="A47:C47"/>
@@ -3825,25 +3846,6 @@
     <mergeCell ref="D51:F51"/>
     <mergeCell ref="A52:C52"/>
     <mergeCell ref="D52:F52"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="D43:F43"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0.35433070866141736" bottom="0" header="0" footer="0"/>
@@ -3853,534 +3855,535 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7121169-D626-4954-A0C3-D0B109C5A29F}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:K18099"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="1" max="2" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="34.28515625" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="92" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4" t="s">
+      <c r="B3" s="94"/>
+      <c r="C3" s="94"/>
+      <c r="D3" s="95" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6" t="s">
+      <c r="A4" s="85"/>
+      <c r="B4" s="85"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="96" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="8"/>
+      <c r="E4" s="97"/>
+      <c r="F4" s="98"/>
     </row>
     <row r="5" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="85" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="11"/>
+      <c r="B5" s="85"/>
+      <c r="C5" s="85"/>
+      <c r="D5" s="86"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="88"/>
     </row>
     <row r="6" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="85" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="12" t="s">
+      <c r="B6" s="85"/>
+      <c r="C6" s="85"/>
+      <c r="D6" s="89" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
+      <c r="E6" s="89"/>
+      <c r="F6" s="89"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
+      <c r="B7" s="90"/>
+      <c r="C7" s="90"/>
+      <c r="D7" s="91"/>
+      <c r="E7" s="91"/>
+      <c r="F7" s="91"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="18"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23" t="s">
+      <c r="C9" s="7"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="24" t="s">
+      <c r="F9" s="10" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="22"/>
-      <c r="E10" s="17" t="s">
+      <c r="D10" s="8"/>
+      <c r="E10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="27" t="s">
+      <c r="F10" s="13" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="28" t="s">
+      <c r="B11" s="3"/>
+      <c r="C11" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="17" t="s">
+      <c r="D11" s="8"/>
+      <c r="E11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="29" t="s">
+      <c r="F11" s="15" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="31"/>
-      <c r="C12" s="28" t="s">
+      <c r="B12" s="17"/>
+      <c r="C12" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="22"/>
-      <c r="E12" s="31" t="s">
+      <c r="D12" s="8"/>
+      <c r="E12" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="27" t="s">
+      <c r="F12" s="13" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="33"/>
-      <c r="D13" s="33"/>
-      <c r="E13" s="34" t="s">
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="34" t="s">
+      <c r="F13" s="19" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="35" t="s">
+      <c r="A14" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="37"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="39" t="s">
+      <c r="C14" s="22"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="39" t="s">
+      <c r="F14" s="24" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="35"/>
-      <c r="B15" s="36"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="35"/>
-      <c r="B16" s="41"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="H16" s="98"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="H16" s="67"/>
     </row>
     <row r="17" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="35"/>
-      <c r="B17" s="44"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
+      <c r="A17" s="20"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
     </row>
     <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="35"/>
-      <c r="B18" s="41"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="45"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="30"/>
     </row>
     <row r="19" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="35"/>
-      <c r="B19" s="46"/>
-      <c r="C19" s="42"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="45"/>
+      <c r="A19" s="20"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="30"/>
     </row>
     <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
-      <c r="B20" s="48"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="50"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="45"/>
-      <c r="I20" s="98"/>
+      <c r="A20" s="32"/>
+      <c r="B20" s="78"/>
+      <c r="C20" s="79"/>
+      <c r="D20" s="80"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="30"/>
+      <c r="I20" s="67"/>
     </row>
     <row r="21" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="47"/>
-      <c r="B21" s="51"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="45"/>
-      <c r="K21" s="98"/>
+      <c r="A21" s="32"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="30"/>
+      <c r="K21" s="67"/>
     </row>
     <row r="22" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="47"/>
-      <c r="B22" s="48"/>
-      <c r="C22" s="49"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="54"/>
+      <c r="A22" s="32"/>
+      <c r="B22" s="78"/>
+      <c r="C22" s="79"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="36"/>
     </row>
     <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="47"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
+      <c r="A23" s="32"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
     </row>
     <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="35"/>
-      <c r="B24" s="57"/>
-      <c r="C24" s="58"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="39"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
     </row>
     <row r="25" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="35"/>
-      <c r="B25" s="57"/>
-      <c r="C25" s="58"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="59"/>
+      <c r="A25" s="20"/>
+      <c r="B25" s="39"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="41"/>
     </row>
     <row r="26" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="35"/>
-      <c r="B26" s="36"/>
-      <c r="C26" s="52"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="59"/>
+      <c r="A26" s="20"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="41"/>
     </row>
     <row r="27" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="35"/>
-      <c r="B27" s="36"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="56"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="60"/>
+      <c r="A27" s="20"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="42"/>
     </row>
     <row r="28" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="35"/>
-      <c r="B28" s="36"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="60"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="42"/>
     </row>
     <row r="29" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="35"/>
-      <c r="B29" s="51"/>
-      <c r="C29" s="61"/>
-      <c r="D29" s="40"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="60"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="33"/>
+      <c r="C29" s="43"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="42"/>
     </row>
     <row r="30" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="35"/>
-      <c r="B30" s="51"/>
-      <c r="C30" s="61"/>
-      <c r="D30" s="56"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="60"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="33"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="42"/>
     </row>
     <row r="31" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="35"/>
-      <c r="B31" s="36"/>
-      <c r="C31" s="61"/>
-      <c r="D31" s="56"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="60"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="42"/>
     </row>
     <row r="32" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="35"/>
-      <c r="B32" s="51"/>
-      <c r="C32" s="61"/>
-      <c r="D32" s="62"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="60"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="33"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="42"/>
     </row>
     <row r="33" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="35"/>
-      <c r="B33" s="36"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="39"/>
-      <c r="F33" s="60"/>
+      <c r="A33" s="20"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="42"/>
     </row>
     <row r="34" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="35"/>
-      <c r="B34" s="48"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="50"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="63"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="78"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="80"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="45"/>
     </row>
     <row r="35" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="35"/>
-      <c r="B35" s="64"/>
-      <c r="C35" s="65"/>
-      <c r="D35" s="66"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="67"/>
+      <c r="A35" s="20"/>
+      <c r="B35" s="46"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="49"/>
     </row>
     <row r="36" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="35"/>
-      <c r="B36" s="68"/>
-      <c r="C36" s="69"/>
-      <c r="D36" s="70"/>
-      <c r="E36" s="71"/>
-      <c r="F36" s="67"/>
+      <c r="A36" s="20"/>
+      <c r="B36" s="50"/>
+      <c r="C36" s="51"/>
+      <c r="D36" s="52"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="49"/>
     </row>
     <row r="37" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="35"/>
-      <c r="B37" s="72"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="70"/>
-      <c r="E37" s="39"/>
-      <c r="F37" s="67"/>
+      <c r="A37" s="20"/>
+      <c r="B37" s="54"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="52"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="49"/>
     </row>
     <row r="38" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="35"/>
-      <c r="B38" s="73"/>
-      <c r="C38" s="74"/>
-      <c r="D38" s="38"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="45"/>
+      <c r="A38" s="20"/>
+      <c r="B38" s="55"/>
+      <c r="C38" s="56"/>
+      <c r="D38" s="23"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="30"/>
     </row>
     <row r="39" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="35"/>
-      <c r="B39" s="36"/>
-      <c r="C39" s="75"/>
-      <c r="D39" s="70"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="45"/>
+      <c r="A39" s="20"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="57"/>
+      <c r="D39" s="52"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="30"/>
     </row>
     <row r="40" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="35"/>
-      <c r="B40" s="76"/>
-      <c r="C40" s="75"/>
-      <c r="D40" s="70"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="45"/>
+      <c r="A40" s="20"/>
+      <c r="B40" s="58"/>
+      <c r="C40" s="57"/>
+      <c r="D40" s="52"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="30"/>
     </row>
     <row r="41" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="35"/>
-      <c r="B41" s="77"/>
-      <c r="C41" s="78"/>
-      <c r="D41" s="79"/>
-      <c r="E41" s="80"/>
-      <c r="F41" s="81"/>
+      <c r="A41" s="20"/>
+      <c r="B41" s="81"/>
+      <c r="C41" s="82"/>
+      <c r="D41" s="83"/>
+      <c r="E41" s="59"/>
+      <c r="F41" s="60"/>
     </row>
     <row r="42" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="35"/>
-      <c r="B42" s="82"/>
-      <c r="C42" s="75"/>
-      <c r="D42" s="70"/>
-      <c r="E42" s="80"/>
-      <c r="F42" s="81"/>
+      <c r="A42" s="20"/>
+      <c r="B42" s="61"/>
+      <c r="C42" s="57"/>
+      <c r="D42" s="52"/>
+      <c r="E42" s="59"/>
+      <c r="F42" s="60"/>
     </row>
     <row r="43" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="83" t="s">
+      <c r="A43" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="B43" s="83"/>
-      <c r="C43" s="83"/>
-      <c r="D43" s="83" t="s">
+      <c r="B43" s="84"/>
+      <c r="C43" s="84"/>
+      <c r="D43" s="84" t="s">
         <v>21</v>
       </c>
-      <c r="E43" s="83"/>
-      <c r="F43" s="83"/>
+      <c r="E43" s="84"/>
+      <c r="F43" s="84"/>
     </row>
     <row r="44" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="84"/>
-      <c r="B44" s="85"/>
-      <c r="C44" s="86"/>
-      <c r="D44" s="85"/>
-      <c r="E44" s="85"/>
-      <c r="F44" s="86"/>
+      <c r="A44" s="62"/>
+      <c r="B44" s="63"/>
+      <c r="C44" s="64"/>
+      <c r="D44" s="63"/>
+      <c r="E44" s="63"/>
+      <c r="F44" s="64"/>
     </row>
     <row r="45" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="15" t="s">
+      <c r="A45" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B45" s="26" t="s">
+      <c r="B45" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="18"/>
-      <c r="D45" s="17" t="s">
+      <c r="C45" s="4"/>
+      <c r="D45" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E45" s="26" t="s">
+      <c r="E45" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="F45" s="87"/>
+      <c r="F45" s="65"/>
     </row>
     <row r="46" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
-      <c r="B46" s="17"/>
-      <c r="C46" s="18"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="18"/>
+      <c r="A46" s="1"/>
+      <c r="B46" s="3"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="4"/>
     </row>
     <row r="47" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="88" t="s">
+      <c r="A47" s="71" t="s">
         <v>24</v>
       </c>
-      <c r="B47" s="89"/>
-      <c r="C47" s="90"/>
-      <c r="D47" s="91" t="s">
+      <c r="B47" s="72"/>
+      <c r="C47" s="73"/>
+      <c r="D47" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="E47" s="91" t="s">
+      <c r="E47" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="F47" s="18"/>
+      <c r="F47" s="4"/>
     </row>
     <row r="48" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="88" t="s">
+      <c r="A48" s="71" t="s">
         <v>27</v>
       </c>
-      <c r="B48" s="89"/>
-      <c r="C48" s="90"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17" t="s">
+      <c r="B48" s="72"/>
+      <c r="C48" s="73"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F48" s="18"/>
+      <c r="F48" s="4"/>
     </row>
     <row r="49" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="15"/>
-      <c r="B49" s="17"/>
-      <c r="C49" s="18"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="18"/>
+      <c r="A49" s="1"/>
+      <c r="B49" s="3"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="4"/>
     </row>
     <row r="50" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="15"/>
-      <c r="B50" s="17"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="17"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="18"/>
+      <c r="A50" s="1"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="4"/>
     </row>
     <row r="51" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="92" t="s">
+      <c r="A51" s="74" t="s">
         <v>42</v>
       </c>
-      <c r="B51" s="93"/>
-      <c r="C51" s="94"/>
-      <c r="D51" s="93" t="s">
+      <c r="B51" s="75"/>
+      <c r="C51" s="76"/>
+      <c r="D51" s="75" t="s">
         <v>44</v>
       </c>
-      <c r="E51" s="93"/>
-      <c r="F51" s="94"/>
+      <c r="E51" s="75"/>
+      <c r="F51" s="76"/>
     </row>
     <row r="52" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="88" t="s">
+      <c r="A52" s="71" t="s">
         <v>30</v>
       </c>
-      <c r="B52" s="89"/>
-      <c r="C52" s="90"/>
-      <c r="D52" s="89" t="s">
+      <c r="B52" s="72"/>
+      <c r="C52" s="73"/>
+      <c r="D52" s="72" t="s">
         <v>31</v>
       </c>
-      <c r="E52" s="89"/>
-      <c r="F52" s="90"/>
+      <c r="E52" s="72"/>
+      <c r="F52" s="73"/>
     </row>
     <row r="53" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="95"/>
-      <c r="B53" s="96"/>
-      <c r="C53" s="97"/>
-      <c r="D53" s="96"/>
-      <c r="E53" s="96"/>
-      <c r="F53" s="97"/>
+      <c r="A53" s="68"/>
+      <c r="B53" s="69"/>
+      <c r="C53" s="70"/>
+      <c r="D53" s="69"/>
+      <c r="E53" s="69"/>
+      <c r="F53" s="70"/>
     </row>
     <row r="54" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6510,6 +6513,25 @@
     <row r="18099" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="D43:F43"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B41:D41"/>
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="D53:F53"/>
     <mergeCell ref="A47:C47"/>
@@ -6518,25 +6540,6 @@
     <mergeCell ref="D51:F51"/>
     <mergeCell ref="A52:C52"/>
     <mergeCell ref="D52:F52"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="D43:F43"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0.35433070866141736" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
fix: improve loader for UI/UX
</commit_message>
<xml_diff>
--- a/procurement_documents/IAR Template.xlsx
+++ b/procurement_documents/IAR Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1882B32E-5EC8-443C-B214-EA64B92EAF73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F189163E-FD55-4883-80D1-84847093A9F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{6CD071E1-92CF-4D3E-842E-C4264179AD1A}"/>
   </bookViews>
@@ -606,7 +606,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -769,161 +769,158 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1363,64 +1360,64 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="112" t="e" vm="1">
+      <c r="A2" s="95" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B2" s="105" t="s">
+      <c r="B2" s="108" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="106"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
+      <c r="C2" s="109"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="109"/>
-      <c r="B3" s="107"/>
-      <c r="C3" s="108"/>
-      <c r="D3" s="100" t="s">
+      <c r="A3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="104" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="71"/>
-      <c r="F3" s="71"/>
+      <c r="E3" s="105"/>
+      <c r="F3" s="105"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="109"/>
-      <c r="B4" s="107"/>
-      <c r="C4" s="108"/>
-      <c r="D4" s="101" t="s">
+      <c r="A4" s="96"/>
+      <c r="B4" s="110"/>
+      <c r="C4" s="111"/>
+      <c r="D4" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="74"/>
-      <c r="F4" s="75"/>
+      <c r="E4" s="106"/>
+      <c r="F4" s="107"/>
     </row>
     <row r="5" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="109"/>
-      <c r="B5" s="107"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="102"/>
-      <c r="E5" s="78"/>
-      <c r="F5" s="79"/>
+      <c r="A5" s="96"/>
+      <c r="B5" s="110"/>
+      <c r="C5" s="111"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="82"/>
+      <c r="F5" s="83"/>
     </row>
     <row r="6" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="109" t="s">
+      <c r="A6" s="96" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="111"/>
-      <c r="C6" s="110"/>
-      <c r="D6" s="103" t="s">
+      <c r="B6" s="97"/>
+      <c r="C6" s="98"/>
+      <c r="D6" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="80"/>
-      <c r="F6" s="80"/>
+      <c r="E6" s="85"/>
+      <c r="F6" s="85"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="113"/>
-      <c r="B7" s="114"/>
-      <c r="C7" s="115"/>
-      <c r="D7" s="104"/>
-      <c r="E7" s="82"/>
-      <c r="F7" s="82"/>
+      <c r="A7" s="99"/>
+      <c r="B7" s="100"/>
+      <c r="C7" s="101"/>
+      <c r="D7" s="86"/>
+      <c r="E7" s="87"/>
+      <c r="F7" s="87"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -1442,7 +1439,7 @@
       <c r="E9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="10"/>
+      <c r="F9" s="118"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -1484,11 +1481,11 @@
       <c r="A13" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="83" t="s">
+      <c r="B13" s="88" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="83"/>
-      <c r="D13" s="83"/>
+      <c r="C13" s="88"/>
+      <c r="D13" s="88"/>
       <c r="E13" s="19" t="s">
         <v>18</v>
       </c>
@@ -1497,186 +1494,186 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="116"/>
+      <c r="A14" s="68"/>
       <c r="B14" s="21"/>
       <c r="C14" s="22"/>
       <c r="D14" s="23"/>
-      <c r="E14" s="118"/>
-      <c r="F14" s="118"/>
+      <c r="E14" s="70"/>
+      <c r="F14" s="70"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="116"/>
+      <c r="A15" s="68"/>
       <c r="B15" s="21"/>
       <c r="C15" s="22"/>
       <c r="D15" s="25"/>
-      <c r="E15" s="118"/>
-      <c r="F15" s="118"/>
+      <c r="E15" s="70"/>
+      <c r="F15" s="70"/>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="116"/>
+      <c r="A16" s="68"/>
       <c r="B16" s="26"/>
       <c r="C16" s="27"/>
       <c r="D16" s="28"/>
-      <c r="E16" s="118"/>
-      <c r="F16" s="118"/>
+      <c r="E16" s="70"/>
+      <c r="F16" s="70"/>
       <c r="H16" s="67"/>
     </row>
     <row r="17" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="116"/>
+      <c r="A17" s="68"/>
       <c r="B17" s="29"/>
       <c r="C17" s="27"/>
       <c r="D17" s="28"/>
-      <c r="E17" s="118"/>
-      <c r="F17" s="118"/>
+      <c r="E17" s="70"/>
+      <c r="F17" s="70"/>
     </row>
     <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="116"/>
+      <c r="A18" s="68"/>
       <c r="B18" s="26"/>
       <c r="C18" s="27"/>
       <c r="D18" s="28"/>
-      <c r="E18" s="118"/>
+      <c r="E18" s="70"/>
       <c r="F18" s="30"/>
     </row>
     <row r="19" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="116"/>
+      <c r="A19" s="68"/>
       <c r="B19" s="31"/>
       <c r="C19" s="27"/>
       <c r="D19" s="28"/>
-      <c r="E19" s="118"/>
+      <c r="E19" s="70"/>
       <c r="F19" s="30"/>
     </row>
     <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="117"/>
-      <c r="B20" s="84"/>
-      <c r="C20" s="85"/>
-      <c r="D20" s="86"/>
-      <c r="E20" s="118"/>
+      <c r="A20" s="69"/>
+      <c r="B20" s="89"/>
+      <c r="C20" s="90"/>
+      <c r="D20" s="91"/>
+      <c r="E20" s="70"/>
       <c r="F20" s="30"/>
       <c r="I20" s="67"/>
     </row>
     <row r="21" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="117"/>
+      <c r="A21" s="69"/>
       <c r="B21" s="33"/>
       <c r="C21" s="34"/>
       <c r="D21" s="35"/>
-      <c r="E21" s="118"/>
+      <c r="E21" s="70"/>
       <c r="F21" s="30"/>
       <c r="K21" s="67"/>
     </row>
     <row r="22" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="117"/>
-      <c r="B22" s="84"/>
-      <c r="C22" s="85"/>
-      <c r="D22" s="86"/>
-      <c r="E22" s="118"/>
+      <c r="A22" s="69"/>
+      <c r="B22" s="89"/>
+      <c r="C22" s="90"/>
+      <c r="D22" s="91"/>
+      <c r="E22" s="70"/>
       <c r="F22" s="36"/>
     </row>
     <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="117"/>
+      <c r="A23" s="69"/>
       <c r="B23" s="26"/>
       <c r="C23" s="37"/>
       <c r="D23" s="38"/>
-      <c r="E23" s="118"/>
-      <c r="F23" s="118"/>
+      <c r="E23" s="70"/>
+      <c r="F23" s="70"/>
     </row>
     <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="116"/>
+      <c r="A24" s="68"/>
       <c r="B24" s="39"/>
       <c r="C24" s="40"/>
       <c r="D24" s="38"/>
-      <c r="E24" s="118"/>
-      <c r="F24" s="118"/>
+      <c r="E24" s="70"/>
+      <c r="F24" s="70"/>
     </row>
     <row r="25" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="116"/>
+      <c r="A25" s="68"/>
       <c r="B25" s="39"/>
       <c r="C25" s="40"/>
       <c r="D25" s="38"/>
-      <c r="E25" s="118"/>
-      <c r="F25" s="119"/>
+      <c r="E25" s="70"/>
+      <c r="F25" s="71"/>
     </row>
     <row r="26" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="116"/>
+      <c r="A26" s="68"/>
       <c r="B26" s="21"/>
       <c r="C26" s="34"/>
       <c r="D26" s="25"/>
-      <c r="E26" s="118"/>
-      <c r="F26" s="119"/>
+      <c r="E26" s="70"/>
+      <c r="F26" s="71"/>
     </row>
     <row r="27" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="116"/>
+      <c r="A27" s="68"/>
       <c r="B27" s="21"/>
       <c r="C27" s="34"/>
       <c r="D27" s="38"/>
-      <c r="E27" s="118"/>
+      <c r="E27" s="70"/>
       <c r="F27" s="42"/>
     </row>
     <row r="28" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="116"/>
+      <c r="A28" s="68"/>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
       <c r="D28" s="25"/>
-      <c r="E28" s="118"/>
+      <c r="E28" s="70"/>
       <c r="F28" s="42"/>
     </row>
     <row r="29" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="116"/>
+      <c r="A29" s="68"/>
       <c r="B29" s="33"/>
       <c r="C29" s="43"/>
       <c r="D29" s="25"/>
-      <c r="E29" s="118"/>
+      <c r="E29" s="70"/>
       <c r="F29" s="42"/>
     </row>
     <row r="30" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="116"/>
+      <c r="A30" s="68"/>
       <c r="B30" s="33"/>
       <c r="C30" s="43"/>
       <c r="D30" s="38"/>
-      <c r="E30" s="118"/>
+      <c r="E30" s="70"/>
       <c r="F30" s="42"/>
     </row>
     <row r="31" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="116"/>
+      <c r="A31" s="68"/>
       <c r="B31" s="21"/>
       <c r="C31" s="43"/>
       <c r="D31" s="38"/>
-      <c r="E31" s="118"/>
+      <c r="E31" s="70"/>
       <c r="F31" s="42"/>
     </row>
     <row r="32" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="116"/>
+      <c r="A32" s="68"/>
       <c r="B32" s="33"/>
       <c r="C32" s="43"/>
       <c r="D32" s="44"/>
-      <c r="E32" s="118"/>
+      <c r="E32" s="70"/>
       <c r="F32" s="42"/>
     </row>
     <row r="33" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="116"/>
+      <c r="A33" s="68"/>
       <c r="B33" s="21"/>
       <c r="C33" s="34"/>
       <c r="D33" s="38"/>
-      <c r="E33" s="118"/>
+      <c r="E33" s="70"/>
       <c r="F33" s="42"/>
     </row>
     <row r="34" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="116"/>
-      <c r="B34" s="84"/>
-      <c r="C34" s="85"/>
-      <c r="D34" s="86"/>
-      <c r="E34" s="118"/>
+      <c r="A34" s="68"/>
+      <c r="B34" s="89"/>
+      <c r="C34" s="90"/>
+      <c r="D34" s="91"/>
+      <c r="E34" s="70"/>
       <c r="F34" s="45"/>
     </row>
     <row r="35" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="116"/>
+      <c r="A35" s="68"/>
       <c r="B35" s="46"/>
       <c r="C35" s="47"/>
       <c r="D35" s="48"/>
-      <c r="E35" s="118"/>
+      <c r="E35" s="70"/>
       <c r="F35" s="49"/>
     </row>
     <row r="36" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="116"/>
+      <c r="A36" s="68"/>
       <c r="B36" s="50"/>
       <c r="C36" s="51"/>
       <c r="D36" s="52"/>
@@ -1684,47 +1681,47 @@
       <c r="F36" s="49"/>
     </row>
     <row r="37" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="116"/>
+      <c r="A37" s="68"/>
       <c r="B37" s="54"/>
       <c r="C37" s="34"/>
       <c r="D37" s="52"/>
-      <c r="E37" s="118"/>
+      <c r="E37" s="70"/>
       <c r="F37" s="49"/>
     </row>
     <row r="38" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="116"/>
+      <c r="A38" s="68"/>
       <c r="B38" s="55"/>
       <c r="C38" s="56"/>
       <c r="D38" s="23"/>
-      <c r="E38" s="118"/>
+      <c r="E38" s="70"/>
       <c r="F38" s="30"/>
     </row>
     <row r="39" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="116"/>
+      <c r="A39" s="68"/>
       <c r="B39" s="21"/>
       <c r="C39" s="57"/>
       <c r="D39" s="52"/>
-      <c r="E39" s="118"/>
+      <c r="E39" s="70"/>
       <c r="F39" s="30"/>
     </row>
     <row r="40" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="116"/>
+      <c r="A40" s="68"/>
       <c r="B40" s="58"/>
       <c r="C40" s="57"/>
       <c r="D40" s="52"/>
-      <c r="E40" s="118"/>
+      <c r="E40" s="70"/>
       <c r="F40" s="30"/>
     </row>
     <row r="41" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="116"/>
-      <c r="B41" s="87"/>
-      <c r="C41" s="88"/>
-      <c r="D41" s="89"/>
+      <c r="A41" s="68"/>
+      <c r="B41" s="92"/>
+      <c r="C41" s="93"/>
+      <c r="D41" s="94"/>
       <c r="E41" s="59"/>
       <c r="F41" s="60"/>
     </row>
     <row r="42" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="116"/>
+      <c r="A42" s="68"/>
       <c r="B42" s="61"/>
       <c r="C42" s="57"/>
       <c r="D42" s="52"/>
@@ -1732,16 +1729,16 @@
       <c r="F42" s="60"/>
     </row>
     <row r="43" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="76" t="s">
+      <c r="A43" s="81" t="s">
         <v>20</v>
       </c>
-      <c r="B43" s="76"/>
-      <c r="C43" s="76"/>
-      <c r="D43" s="76" t="s">
+      <c r="B43" s="81"/>
+      <c r="C43" s="81"/>
+      <c r="D43" s="81" t="s">
         <v>21</v>
       </c>
-      <c r="E43" s="76"/>
-      <c r="F43" s="76"/>
+      <c r="E43" s="81"/>
+      <c r="F43" s="81"/>
     </row>
     <row r="44" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="62"/>
@@ -1772,11 +1769,11 @@
       <c r="F46" s="4"/>
     </row>
     <row r="47" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="93" t="s">
+      <c r="A47" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B47" s="94"/>
-      <c r="C47" s="95"/>
+      <c r="B47" s="76"/>
+      <c r="C47" s="77"/>
       <c r="D47" s="66" t="s">
         <v>25</v>
       </c>
@@ -1786,11 +1783,11 @@
       <c r="F47" s="4"/>
     </row>
     <row r="48" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="93" t="s">
+      <c r="A48" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="B48" s="94"/>
-      <c r="C48" s="95"/>
+      <c r="B48" s="76"/>
+      <c r="C48" s="77"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3" t="s">
         <v>28</v>
@@ -1814,34 +1811,34 @@
       <c r="F50" s="4"/>
     </row>
     <row r="51" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="96"/>
-      <c r="B51" s="97"/>
-      <c r="C51" s="98"/>
-      <c r="D51" s="97" t="s">
+      <c r="A51" s="78"/>
+      <c r="B51" s="79"/>
+      <c r="C51" s="80"/>
+      <c r="D51" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="E51" s="97"/>
-      <c r="F51" s="98"/>
+      <c r="E51" s="79"/>
+      <c r="F51" s="80"/>
     </row>
     <row r="52" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="93" t="s">
+      <c r="A52" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="B52" s="94"/>
-      <c r="C52" s="95"/>
-      <c r="D52" s="94" t="s">
+      <c r="B52" s="76"/>
+      <c r="C52" s="77"/>
+      <c r="D52" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="E52" s="94"/>
-      <c r="F52" s="95"/>
+      <c r="E52" s="76"/>
+      <c r="F52" s="77"/>
     </row>
     <row r="53" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="90"/>
-      <c r="B53" s="91"/>
-      <c r="C53" s="92"/>
-      <c r="D53" s="91"/>
-      <c r="E53" s="91"/>
-      <c r="F53" s="92"/>
+      <c r="A53" s="72"/>
+      <c r="B53" s="73"/>
+      <c r="C53" s="74"/>
+      <c r="D53" s="73"/>
+      <c r="E53" s="73"/>
+      <c r="F53" s="74"/>
     </row>
     <row r="54" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3971,14 +3968,6 @@
     <row r="18099" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="D52:F52"/>
     <mergeCell ref="A43:C43"/>
     <mergeCell ref="D43:F43"/>
     <mergeCell ref="D5:F5"/>
@@ -3995,6 +3984,14 @@
     <mergeCell ref="D3:F3"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="B2:C5"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="D52:F52"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0.35433070866141736" bottom="0" header="0" footer="0"/>
@@ -4016,68 +4013,68 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="115" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
+      <c r="B2" s="115"/>
+      <c r="C2" s="115"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="70" t="s">
+      <c r="A3" s="116" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="70"/>
-      <c r="C3" s="70"/>
-      <c r="D3" s="71" t="s">
+      <c r="B3" s="116"/>
+      <c r="C3" s="116"/>
+      <c r="D3" s="105" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="71"/>
-      <c r="F3" s="71"/>
+      <c r="E3" s="105"/>
+      <c r="F3" s="105"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="72"/>
-      <c r="B4" s="72"/>
-      <c r="C4" s="72"/>
-      <c r="D4" s="73" t="s">
+      <c r="A4" s="112"/>
+      <c r="B4" s="112"/>
+      <c r="C4" s="112"/>
+      <c r="D4" s="117" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="74"/>
-      <c r="F4" s="75"/>
+      <c r="E4" s="106"/>
+      <c r="F4" s="107"/>
     </row>
     <row r="5" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="72" t="s">
+      <c r="A5" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="72"/>
-      <c r="C5" s="72"/>
-      <c r="D5" s="77"/>
-      <c r="E5" s="78"/>
-      <c r="F5" s="79"/>
+      <c r="B5" s="112"/>
+      <c r="C5" s="112"/>
+      <c r="D5" s="113"/>
+      <c r="E5" s="82"/>
+      <c r="F5" s="83"/>
     </row>
     <row r="6" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="72" t="s">
+      <c r="A6" s="112" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="72"/>
-      <c r="C6" s="72"/>
-      <c r="D6" s="80" t="s">
+      <c r="B6" s="112"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="85" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="80"/>
-      <c r="F6" s="80"/>
+      <c r="E6" s="85"/>
+      <c r="F6" s="85"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="81" t="s">
+      <c r="A7" s="114" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="81"/>
-      <c r="C7" s="81"/>
-      <c r="D7" s="82"/>
-      <c r="E7" s="82"/>
-      <c r="F7" s="82"/>
+      <c r="B7" s="114"/>
+      <c r="C7" s="114"/>
+      <c r="D7" s="87"/>
+      <c r="E7" s="87"/>
+      <c r="F7" s="87"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -4161,11 +4158,11 @@
       <c r="A13" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="83" t="s">
+      <c r="B13" s="88" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="83"/>
-      <c r="D13" s="83"/>
+      <c r="C13" s="88"/>
+      <c r="D13" s="88"/>
       <c r="E13" s="19" t="s">
         <v>18</v>
       </c>
@@ -4232,9 +4229,9 @@
     </row>
     <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="32"/>
-      <c r="B20" s="84"/>
-      <c r="C20" s="85"/>
-      <c r="D20" s="86"/>
+      <c r="B20" s="89"/>
+      <c r="C20" s="90"/>
+      <c r="D20" s="91"/>
       <c r="E20" s="24"/>
       <c r="F20" s="30"/>
       <c r="I20" s="67"/>
@@ -4250,9 +4247,9 @@
     </row>
     <row r="22" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="32"/>
-      <c r="B22" s="84"/>
-      <c r="C22" s="85"/>
-      <c r="D22" s="86"/>
+      <c r="B22" s="89"/>
+      <c r="C22" s="90"/>
+      <c r="D22" s="91"/>
       <c r="E22" s="24"/>
       <c r="F22" s="36"/>
     </row>
@@ -4346,9 +4343,9 @@
     </row>
     <row r="34" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="20"/>
-      <c r="B34" s="84"/>
-      <c r="C34" s="85"/>
-      <c r="D34" s="86"/>
+      <c r="B34" s="89"/>
+      <c r="C34" s="90"/>
+      <c r="D34" s="91"/>
       <c r="E34" s="24"/>
       <c r="F34" s="45"/>
     </row>
@@ -4402,9 +4399,9 @@
     </row>
     <row r="41" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="20"/>
-      <c r="B41" s="87"/>
-      <c r="C41" s="88"/>
-      <c r="D41" s="89"/>
+      <c r="B41" s="92"/>
+      <c r="C41" s="93"/>
+      <c r="D41" s="94"/>
       <c r="E41" s="59"/>
       <c r="F41" s="60"/>
     </row>
@@ -4417,16 +4414,16 @@
       <c r="F42" s="60"/>
     </row>
     <row r="43" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="76" t="s">
+      <c r="A43" s="81" t="s">
         <v>20</v>
       </c>
-      <c r="B43" s="76"/>
-      <c r="C43" s="76"/>
-      <c r="D43" s="76" t="s">
+      <c r="B43" s="81"/>
+      <c r="C43" s="81"/>
+      <c r="D43" s="81" t="s">
         <v>21</v>
       </c>
-      <c r="E43" s="76"/>
-      <c r="F43" s="76"/>
+      <c r="E43" s="81"/>
+      <c r="F43" s="81"/>
     </row>
     <row r="44" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="62"/>
@@ -4461,11 +4458,11 @@
       <c r="F46" s="4"/>
     </row>
     <row r="47" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="93" t="s">
+      <c r="A47" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B47" s="94"/>
-      <c r="C47" s="95"/>
+      <c r="B47" s="76"/>
+      <c r="C47" s="77"/>
       <c r="D47" s="66" t="s">
         <v>25</v>
       </c>
@@ -4475,11 +4472,11 @@
       <c r="F47" s="4"/>
     </row>
     <row r="48" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="93" t="s">
+      <c r="A48" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="B48" s="94"/>
-      <c r="C48" s="95"/>
+      <c r="B48" s="76"/>
+      <c r="C48" s="77"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3" t="s">
         <v>28</v>
@@ -4503,36 +4500,36 @@
       <c r="F50" s="4"/>
     </row>
     <row r="51" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="96" t="s">
+      <c r="A51" s="78" t="s">
         <v>42</v>
       </c>
-      <c r="B51" s="97"/>
-      <c r="C51" s="98"/>
-      <c r="D51" s="97" t="s">
+      <c r="B51" s="79"/>
+      <c r="C51" s="80"/>
+      <c r="D51" s="79" t="s">
         <v>44</v>
       </c>
-      <c r="E51" s="97"/>
-      <c r="F51" s="98"/>
+      <c r="E51" s="79"/>
+      <c r="F51" s="80"/>
     </row>
     <row r="52" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="93" t="s">
+      <c r="A52" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="B52" s="94"/>
-      <c r="C52" s="95"/>
-      <c r="D52" s="94" t="s">
+      <c r="B52" s="76"/>
+      <c r="C52" s="77"/>
+      <c r="D52" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="E52" s="94"/>
-      <c r="F52" s="95"/>
+      <c r="E52" s="76"/>
+      <c r="F52" s="77"/>
     </row>
     <row r="53" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="90"/>
-      <c r="B53" s="91"/>
-      <c r="C53" s="92"/>
-      <c r="D53" s="91"/>
-      <c r="E53" s="91"/>
-      <c r="F53" s="92"/>
+      <c r="A53" s="72"/>
+      <c r="B53" s="73"/>
+      <c r="C53" s="74"/>
+      <c r="D53" s="73"/>
+      <c r="E53" s="73"/>
+      <c r="F53" s="74"/>
     </row>
     <row r="54" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6662,14 +6659,12 @@
     <row r="18099" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
     <mergeCell ref="A43:C43"/>
     <mergeCell ref="D43:F43"/>
     <mergeCell ref="A5:C5"/>
@@ -6683,12 +6678,14 @@
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B41:D41"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="D52:F52"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0.35433070866141736" bottom="0" header="0" footer="0"/>

</xml_diff>